<commit_message>
feat: show cover art and online book details
- Add cover art and external book metadata to the book dialog.
</commit_message>
<xml_diff>
--- a/public/data/template.xlsx
+++ b/public/data/template.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">書名</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t xml:space="preserve">藏書位置</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISBN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">封面連結</t>
   </si>
   <si>
     <t xml:space="preserve">走在夢的路上</t>
@@ -177,6 +183,8 @@
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -216,81 +224,87 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J2" s="0">
         <v>320</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J3" s="0">
         <v>250</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: show cover art and online book details in the book dialog
</commit_message>
<xml_diff>
--- a/public/data/template.xlsx
+++ b/public/data/template.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">書名</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t xml:space="preserve">藏書位置</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISBN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">封面連結</t>
   </si>
   <si>
     <t xml:space="preserve">走在夢的路上</t>
@@ -177,6 +183,8 @@
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -216,81 +224,87 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J2" s="0">
         <v>320</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J3" s="0">
         <v>250</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: page size, display settings, and no book images
- Add URL-persisted page-size controls.
- Add browser-persisted theme, text-size, and page-width settings.
- Remove book images and retailer search links.
- Keep the unused cover_url column for schema compatibility.
</commit_message>
<xml_diff>
--- a/public/data/template.xlsx
+++ b/public/data/template.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">書名</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t xml:space="preserve">ISBN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">封面連結</t>
   </si>
   <si>
     <t xml:space="preserve">走在夢的路上</t>
@@ -184,7 +181,6 @@
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -227,84 +223,81 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="0" t="s">
+      <c r="E2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>20</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>21</v>
       </c>
       <c r="J2" s="0">
         <v>320</v>
       </c>
       <c r="K2" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" s="0" t="s">
         <v>22</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E3" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="G3" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>31</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>32</v>
       </c>
       <c r="J3" s="0">
         <v>250</v>
       </c>
       <c r="K3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" s="0" t="s">
         <v>33</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>